<commit_message>
test case postiive 2 edit
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/02/data/new-rule-positive-2.xlsx
+++ b/rules/NEW-RULE/positive/02/data/new-rule-positive-2.xlsx
@@ -494,7 +494,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -706,9 +706,44 @@
         <v>2018-12-21</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="4" t="str">
+        <v>TS</v>
+      </c>
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="4" t="str">
+        <v>AGEMIN</v>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v>Minimum Age</v>
+      </c>
+      <c r="G7" s="4">
+        <v>18</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="I7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="J7" s="4" t="str">
+        <v>CDISC</v>
+      </c>
+      <c r="K7" s="4" t="str">
+        <v>2018-12-21</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>